<commit_message>
v0.7 (FIRST STABLE BUILD)
Finally, a stable build. Still some stuff needs to be added, but everything that exists has been properly stress tested. Minor issues still exist, of course, and will be ironed out asap.
</commit_message>
<xml_diff>
--- a/skiltracker-main.xlsx
+++ b/skiltracker-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Documents\SkilTracker\SkilTracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{631396B4-2753-4628-B84B-F645D85DEDB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC9395C-8E6F-4D9B-ABCA-76FB987FE52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ID" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>ID</t>
   </si>
@@ -65,87 +65,6 @@
     <t>Cat3e</t>
   </si>
   <si>
-    <t>RDR001</t>
-  </si>
-  <si>
-    <t>Planning</t>
-  </si>
-  <si>
-    <t>Gunslinging</t>
-  </si>
-  <si>
-    <t>Heists</t>
-  </si>
-  <si>
-    <t>Fashion</t>
-  </si>
-  <si>
-    <t>Warfare</t>
-  </si>
-  <si>
-    <t>History</t>
-  </si>
-  <si>
-    <t>Music</t>
-  </si>
-  <si>
-    <t>Diplomacy</t>
-  </si>
-  <si>
-    <t>RDR002</t>
-  </si>
-  <si>
-    <t>Capacity</t>
-  </si>
-  <si>
-    <t>Reading</t>
-  </si>
-  <si>
-    <t>Teaching</t>
-  </si>
-  <si>
-    <t>RDR003</t>
-  </si>
-  <si>
-    <t>Main Character</t>
-  </si>
-  <si>
-    <t>Horseback Riding</t>
-  </si>
-  <si>
-    <t>Native Affairs</t>
-  </si>
-  <si>
-    <t>Foraging</t>
-  </si>
-  <si>
-    <t>Hunting</t>
-  </si>
-  <si>
-    <t>Horse Care</t>
-  </si>
-  <si>
-    <t>Childcare</t>
-  </si>
-  <si>
-    <t>Management</t>
-  </si>
-  <si>
-    <t>RDR004</t>
-  </si>
-  <si>
-    <t>Family</t>
-  </si>
-  <si>
-    <t>Gang Warfare</t>
-  </si>
-  <si>
-    <t>RDR005</t>
-  </si>
-  <si>
-    <t>Motherhood</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -156,48 +75,6 @@
   </si>
   <si>
     <t>Sector</t>
-  </si>
-  <si>
-    <t>Dutch</t>
-  </si>
-  <si>
-    <t>Van der Linde</t>
-  </si>
-  <si>
-    <t>Leadership</t>
-  </si>
-  <si>
-    <t>Hosea</t>
-  </si>
-  <si>
-    <t>Matthews</t>
-  </si>
-  <si>
-    <t>Arthur</t>
-  </si>
-  <si>
-    <t>Morgan</t>
-  </si>
-  <si>
-    <t>Enforcement</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Marston</t>
-  </si>
-  <si>
-    <t>Abigail</t>
-  </si>
-  <si>
-    <t>Roberts</t>
-  </si>
-  <si>
-    <t>Support</t>
-  </si>
-  <si>
-    <t>Theft</t>
   </si>
 </sst>
 </file>
@@ -569,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.375" bestFit="1" customWidth="1"/>
@@ -581,101 +458,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D2">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D3">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -690,7 +482,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -732,121 +524,6 @@
       </c>
       <c r="M1" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>